<commit_message>
Week 2 evals processed. Week 3 evals generated.
</commit_message>
<xml_diff>
--- a/Function 1/evals.xlsx
+++ b/Function 1/evals.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone Project\Function 1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A77A8F20-A7FA-4750-9459-0E56BEE57385}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{103DB947-CADE-4235-9127-6C15B6B84BD4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -82,14 +82,14 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -377,198 +377,212 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1" t="s">
+      <c r="E2" s="3"/>
+      <c r="F2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1" t="s">
+      <c r="G2" s="3"/>
+      <c r="H2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="1"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="2">
+      <c r="B3" s="4">
         <v>1</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2">
+      <c r="C3" s="4"/>
+      <c r="D3" s="4">
         <v>0.73278699999999997</v>
       </c>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2">
+      <c r="E3" s="4"/>
+      <c r="F3" s="4">
         <v>0.73318099999999997</v>
       </c>
-      <c r="G3" s="2"/>
+      <c r="G3" s="4"/>
       <c r="H3" s="5">
         <v>3.5897238714370398E-16</v>
       </c>
-      <c r="I3" s="2"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
+      <c r="B4" s="4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4">
+        <v>0.45</v>
+      </c>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4">
+        <v>-5.8471552540567497E-6</v>
+      </c>
+      <c r="I4" s="4"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
+      <c r="B5" s="4">
+        <v>3</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4">
+        <v>0.71610380492128201</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4">
+        <v>0.73107980911083703</v>
+      </c>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="52">
@@ -577,34 +591,15 @@
     <mergeCell ref="H14:I14"/>
     <mergeCell ref="F13:G13"/>
     <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
     <mergeCell ref="H4:I4"/>
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="H7:I7"/>
     <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
@@ -612,7 +607,10 @@
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
     <mergeCell ref="D14:E14"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="D4:E4"/>
@@ -620,10 +618,26 @@
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F2:G2"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
processed week 3 evals.
</commit_message>
<xml_diff>
--- a/Function 1/evals.xlsx
+++ b/Function 1/evals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D8ACEE7-AED4-4793-B9B8-4603FE682ECC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16704919-DC14-4EA4-A835-E113AC9587EA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,10 +84,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -377,208 +377,212 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="4"/>
+      <c r="D2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
+      <c r="E2" s="4"/>
+      <c r="F2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3" t="s">
+      <c r="G2" s="4"/>
+      <c r="H2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="3"/>
+      <c r="I2" s="4"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="4">
+      <c r="B3" s="3">
         <v>1</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3">
         <v>0.73278699999999997</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4">
+      <c r="E3" s="3"/>
+      <c r="F3" s="3">
         <v>0.73318099999999997</v>
       </c>
-      <c r="G3" s="4"/>
+      <c r="G3" s="3"/>
       <c r="H3" s="5">
         <v>3.5897238714370398E-16</v>
       </c>
-      <c r="I3" s="4"/>
+      <c r="I3" s="3"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>2</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4">
+      <c r="C4" s="3"/>
+      <c r="D4" s="3">
         <v>0.5</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4">
+      <c r="E4" s="3"/>
+      <c r="F4" s="3">
         <v>0.45</v>
       </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4">
+      <c r="G4" s="3"/>
+      <c r="H4" s="3">
         <v>-5.8471552540567497E-6</v>
       </c>
-      <c r="I4" s="4"/>
+      <c r="I4" s="3"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="4">
+      <c r="B5" s="3">
         <v>3</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4">
+      <c r="C5" s="3"/>
+      <c r="D5" s="3">
         <v>0.71610380492128201</v>
       </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4">
+      <c r="E5" s="3"/>
+      <c r="F5" s="3">
         <v>0.73107980911083703</v>
       </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="5">
+        <v>2.4917657838054898E-13</v>
+      </c>
+      <c r="I5" s="3"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
+      <c r="B6" s="3">
+        <v>4</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
@@ -586,42 +590,6 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
@@ -638,6 +606,42 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="F7:G7"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
added query formatting and sent week 4 queries.
</commit_message>
<xml_diff>
--- a/Function 1/evals.xlsx
+++ b/Function 1/evals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16704919-DC14-4EA4-A835-E113AC9587EA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E47D43-7761-4741-B3C0-5FB9E6F70FE2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,10 +84,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -377,212 +377,216 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4" t="s">
+      <c r="E2" s="3"/>
+      <c r="F2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4" t="s">
+      <c r="G2" s="3"/>
+      <c r="H2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="4"/>
+      <c r="I2" s="3"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="3">
+      <c r="B3" s="4">
         <v>1</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3">
+      <c r="C3" s="4"/>
+      <c r="D3" s="4">
         <v>0.73278699999999997</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3">
+      <c r="E3" s="4"/>
+      <c r="F3" s="4">
         <v>0.73318099999999997</v>
       </c>
-      <c r="G3" s="3"/>
+      <c r="G3" s="4"/>
       <c r="H3" s="5">
         <v>3.5897238714370398E-16</v>
       </c>
-      <c r="I3" s="3"/>
+      <c r="I3" s="4"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="3">
+      <c r="B4" s="4">
         <v>2</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3">
+      <c r="C4" s="4"/>
+      <c r="D4" s="4">
         <v>0.5</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3">
+      <c r="E4" s="4"/>
+      <c r="F4" s="4">
         <v>0.45</v>
       </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3">
+      <c r="G4" s="4"/>
+      <c r="H4" s="4">
         <v>-5.8471552540567497E-6</v>
       </c>
-      <c r="I4" s="3"/>
+      <c r="I4" s="4"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="3">
+      <c r="B5" s="4">
         <v>3</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3">
+      <c r="C5" s="4"/>
+      <c r="D5" s="4">
         <v>0.71610380492128201</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3">
+      <c r="E5" s="4"/>
+      <c r="F5" s="4">
         <v>0.73107980911083703</v>
       </c>
-      <c r="G5" s="3"/>
+      <c r="G5" s="4"/>
       <c r="H5" s="5">
         <v>2.4917657838054898E-13</v>
       </c>
-      <c r="I5" s="3"/>
+      <c r="I5" s="4"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B6" s="3">
+      <c r="B6" s="4">
         <v>4</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4">
+        <v>0.70174915499430002</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4">
+        <v>0.72858430442151101</v>
+      </c>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
@@ -590,6 +594,42 @@
     </row>
   </sheetData>
   <mergeCells count="52">
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
@@ -606,42 +646,6 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="F7:G7"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
generating week 5 queries, commit (1/2).
</commit_message>
<xml_diff>
--- a/Function 1/evals.xlsx
+++ b/Function 1/evals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E47D43-7761-4741-B3C0-5FB9E6F70FE2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD1D4ED8-F3CE-47FA-A470-3AD9766C34BD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,13 +84,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -377,216 +377,224 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="5"/>
+      <c r="D2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
+      <c r="E2" s="5"/>
+      <c r="F2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3" t="s">
+      <c r="G2" s="5"/>
+      <c r="H2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="3"/>
+      <c r="I2" s="5"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="4">
+      <c r="B3" s="3">
         <v>1</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3">
         <v>0.73278699999999997</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4">
+      <c r="E3" s="3"/>
+      <c r="F3" s="3">
         <v>0.73318099999999997</v>
       </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="5">
+      <c r="G3" s="3"/>
+      <c r="H3" s="4">
         <v>3.5897238714370398E-16</v>
       </c>
-      <c r="I3" s="4"/>
+      <c r="I3" s="3"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>2</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4">
+      <c r="C4" s="3"/>
+      <c r="D4" s="3">
         <v>0.5</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4">
+      <c r="E4" s="3"/>
+      <c r="F4" s="3">
         <v>0.45</v>
       </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4">
+      <c r="G4" s="3"/>
+      <c r="H4" s="3">
         <v>-5.8471552540567497E-6</v>
       </c>
-      <c r="I4" s="4"/>
+      <c r="I4" s="3"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="4">
+      <c r="B5" s="3">
         <v>3</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4">
+      <c r="C5" s="3"/>
+      <c r="D5" s="3">
         <v>0.71610380492128201</v>
       </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4">
+      <c r="E5" s="3"/>
+      <c r="F5" s="3">
         <v>0.73107980911083703</v>
       </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="5">
+      <c r="G5" s="3"/>
+      <c r="H5" s="4">
         <v>2.4917657838054898E-13</v>
       </c>
-      <c r="I5" s="4"/>
+      <c r="I5" s="3"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <v>4</v>
       </c>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4">
+      <c r="C6" s="3"/>
+      <c r="D6" s="3">
         <v>0.70174915499430002</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4">
+      <c r="E6" s="3"/>
+      <c r="F6" s="3">
         <v>0.72858430442151101</v>
       </c>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="4">
+        <v>2.66967348318954E-11</v>
+      </c>
+      <c r="I6" s="3"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
+      <c r="B7" s="3">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3">
+        <v>0.69774526461712905</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3">
+        <v>0.72787423209350399</v>
+      </c>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
@@ -594,42 +602,6 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
@@ -646,6 +618,42 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="F7:G7"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
week 6 queries generated.
</commit_message>
<xml_diff>
--- a/Function 1/evals.xlsx
+++ b/Function 1/evals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD1D4ED8-F3CE-47FA-A470-3AD9766C34BD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6628519D-6E17-479A-94E1-1128F95E3709}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -397,10 +397,10 @@
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="3">
+      <c r="B3" s="5">
         <v>1</v>
       </c>
-      <c r="C3" s="3"/>
+      <c r="C3" s="5"/>
       <c r="D3" s="3">
         <v>0.73278699999999997</v>
       </c>
@@ -417,10 +417,10 @@
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="3">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="3"/>
+      <c r="C4" s="5"/>
       <c r="D4" s="3">
         <v>0.5</v>
       </c>
@@ -439,10 +439,10 @@
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="3">
+      <c r="B5" s="5">
         <v>3</v>
       </c>
-      <c r="C5" s="3"/>
+      <c r="C5" s="5"/>
       <c r="D5" s="3">
         <v>0.71610380492128201</v>
       </c>
@@ -461,10 +461,10 @@
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B6" s="3">
+      <c r="B6" s="5">
         <v>4</v>
       </c>
-      <c r="C6" s="3"/>
+      <c r="C6" s="5"/>
       <c r="D6" s="3">
         <v>0.70174915499430002</v>
       </c>
@@ -483,10 +483,10 @@
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="3">
+      <c r="B7" s="5">
         <v>5</v>
       </c>
-      <c r="C7" s="3"/>
+      <c r="C7" s="5"/>
       <c r="D7" s="3">
         <v>0.69774526461712905</v>
       </c>
@@ -495,7 +495,9 @@
         <v>0.72787423209350399</v>
       </c>
       <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
+      <c r="H7" s="4">
+        <v>8.2021938139919396E-11</v>
+      </c>
       <c r="I7" s="3"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
@@ -503,11 +505,17 @@
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+      <c r="B8" s="5">
+        <v>6</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="3">
+        <v>0.69108273489459604</v>
+      </c>
       <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
+      <c r="F8" s="3">
+        <v>0.72641993605285105</v>
+      </c>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>

</xml_diff>

<commit_message>
generating week 6 queries (1/2)
</commit_message>
<xml_diff>
--- a/Function 1/evals.xlsx
+++ b/Function 1/evals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6628519D-6E17-479A-94E1-1128F95E3709}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C1189A-2B3C-433A-9E65-A6CE012D5808}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,13 +84,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -377,232 +377,240 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5" t="s">
+      <c r="E2" s="3"/>
+      <c r="F2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5" t="s">
+      <c r="G2" s="3"/>
+      <c r="H2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="5"/>
+      <c r="I2" s="3"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="5">
+      <c r="B3" s="3">
         <v>1</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="3">
+      <c r="C3" s="3"/>
+      <c r="D3" s="4">
         <v>0.73278699999999997</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3">
+      <c r="E3" s="4"/>
+      <c r="F3" s="4">
         <v>0.73318099999999997</v>
       </c>
-      <c r="G3" s="3"/>
-      <c r="H3" s="4">
+      <c r="G3" s="4"/>
+      <c r="H3" s="5">
         <v>3.5897238714370398E-16</v>
       </c>
-      <c r="I3" s="3"/>
+      <c r="I3" s="4"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="5">
+      <c r="B4" s="3">
         <v>2</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="3">
+      <c r="C4" s="3"/>
+      <c r="D4" s="4">
         <v>0.5</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3">
+      <c r="E4" s="4"/>
+      <c r="F4" s="4">
         <v>0.45</v>
       </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3">
+      <c r="G4" s="4"/>
+      <c r="H4" s="5">
         <v>-5.8471552540567497E-6</v>
       </c>
-      <c r="I4" s="3"/>
+      <c r="I4" s="4"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="5">
+      <c r="B5" s="3">
         <v>3</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="3">
+      <c r="C5" s="3"/>
+      <c r="D5" s="4">
         <v>0.71610380492128201</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3">
+      <c r="E5" s="4"/>
+      <c r="F5" s="4">
         <v>0.73107980911083703</v>
       </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="4">
+      <c r="G5" s="4"/>
+      <c r="H5" s="5">
         <v>2.4917657838054898E-13</v>
       </c>
-      <c r="I5" s="3"/>
+      <c r="I5" s="4"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B6" s="5">
+      <c r="B6" s="3">
         <v>4</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="3">
+      <c r="C6" s="3"/>
+      <c r="D6" s="4">
         <v>0.70174915499430002</v>
       </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3">
+      <c r="E6" s="4"/>
+      <c r="F6" s="4">
         <v>0.72858430442151101</v>
       </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="4">
+      <c r="G6" s="4"/>
+      <c r="H6" s="5">
         <v>2.66967348318954E-11</v>
       </c>
-      <c r="I6" s="3"/>
+      <c r="I6" s="4"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="5">
+      <c r="B7" s="3">
         <v>5</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="3">
+      <c r="C7" s="3"/>
+      <c r="D7" s="4">
         <v>0.69774526461712905</v>
       </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3">
+      <c r="E7" s="4"/>
+      <c r="F7" s="4">
         <v>0.72787423209350399</v>
       </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="4">
+      <c r="G7" s="4"/>
+      <c r="H7" s="5">
         <v>8.2021938139919396E-11</v>
       </c>
-      <c r="I7" s="3"/>
+      <c r="I7" s="4"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="5">
+      <c r="B8" s="3">
         <v>6</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="3">
+      <c r="C8" s="3"/>
+      <c r="D8" s="4">
         <v>0.69108273489459604</v>
       </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3">
+      <c r="E8" s="4"/>
+      <c r="F8" s="4">
         <v>0.72641993605285105</v>
       </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="5">
+        <v>4.8363240034292804E-10</v>
+      </c>
+      <c r="I8" s="4"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="3"/>
+      <c r="B9" s="3">
+        <v>7</v>
+      </c>
       <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
+      <c r="D9" s="4">
+        <v>0.68231104396327502</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4">
+        <v>0.72440711698077198</v>
+      </c>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
@@ -610,6 +618,42 @@
     </row>
   </sheetData>
   <mergeCells count="52">
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
@@ -626,42 +670,6 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="F7:G7"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
week 7 queries generated (1/2).
</commit_message>
<xml_diff>
--- a/Function 1/evals.xlsx
+++ b/Function 1/evals.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C1189A-2B3C-433A-9E65-A6CE012D5808}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E37FB250-F364-4613-AFE8-D52D19B4C019}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -84,13 +84,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -374,243 +374,251 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:M14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="3" t="s">
+    <row r="2" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="5"/>
+      <c r="D2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
+      <c r="E2" s="5"/>
+      <c r="F2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3" t="s">
+      <c r="G2" s="5"/>
+      <c r="H2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="3"/>
+      <c r="I2" s="5"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="3">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B3" s="5">
         <v>1</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="4">
+      <c r="C3" s="5"/>
+      <c r="D3" s="3">
         <v>0.73278699999999997</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4">
+      <c r="E3" s="3"/>
+      <c r="F3" s="3">
         <v>0.73318099999999997</v>
       </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="5">
+      <c r="G3" s="3"/>
+      <c r="H3" s="4">
         <v>3.5897238714370398E-16</v>
       </c>
-      <c r="I3" s="4"/>
+      <c r="I3" s="3"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="3">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="4">
+      <c r="C4" s="5"/>
+      <c r="D4" s="3">
         <v>0.5</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4">
+      <c r="E4" s="3"/>
+      <c r="F4" s="3">
         <v>0.45</v>
       </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="5">
+      <c r="G4" s="3"/>
+      <c r="H4" s="4">
         <v>-5.8471552540567497E-6</v>
       </c>
-      <c r="I4" s="4"/>
+      <c r="I4" s="3"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="3">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B5" s="5">
         <v>3</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="4">
+      <c r="C5" s="5"/>
+      <c r="D5" s="3">
         <v>0.71610380492128201</v>
       </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4">
+      <c r="E5" s="3"/>
+      <c r="F5" s="3">
         <v>0.73107980911083703</v>
       </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="5">
+      <c r="G5" s="3"/>
+      <c r="H5" s="4">
         <v>2.4917657838054898E-13</v>
       </c>
-      <c r="I5" s="4"/>
+      <c r="I5" s="3"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B6" s="3">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B6" s="5">
         <v>4</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="4">
+      <c r="C6" s="5"/>
+      <c r="D6" s="3">
         <v>0.70174915499430002</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4">
+      <c r="E6" s="3"/>
+      <c r="F6" s="3">
         <v>0.72858430442151101</v>
       </c>
-      <c r="G6" s="4"/>
-      <c r="H6" s="5">
+      <c r="G6" s="3"/>
+      <c r="H6" s="4">
         <v>2.66967348318954E-11</v>
       </c>
-      <c r="I6" s="4"/>
+      <c r="I6" s="3"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="3">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B7" s="5">
         <v>5</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="4">
+      <c r="C7" s="5"/>
+      <c r="D7" s="3">
         <v>0.69774526461712905</v>
       </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4">
+      <c r="E7" s="3"/>
+      <c r="F7" s="3">
         <v>0.72787423209350399</v>
       </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="5">
+      <c r="G7" s="3"/>
+      <c r="H7" s="4">
         <v>8.2021938139919396E-11</v>
       </c>
-      <c r="I7" s="4"/>
+      <c r="I7" s="3"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="3">
+    <row r="8" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B8" s="5">
         <v>6</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="4">
+      <c r="C8" s="5"/>
+      <c r="D8" s="3">
         <v>0.69108273489459604</v>
       </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4">
+      <c r="E8" s="3"/>
+      <c r="F8" s="3">
         <v>0.72641993605285105</v>
       </c>
-      <c r="G8" s="4"/>
-      <c r="H8" s="5">
+      <c r="G8" s="3"/>
+      <c r="H8" s="4">
         <v>4.8363240034292804E-10</v>
       </c>
-      <c r="I8" s="4"/>
+      <c r="I8" s="3"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="3">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B9" s="5">
         <v>7</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="4">
+      <c r="C9" s="5"/>
+      <c r="D9" s="3">
         <v>0.68231104396327502</v>
       </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4">
+      <c r="E9" s="3"/>
+      <c r="F9" s="3">
         <v>0.72440711698077198</v>
       </c>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="4">
+        <v>3.3931989655218898E-9</v>
+      </c>
+      <c r="I9" s="3"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
     </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B10" s="5">
+        <v>8</v>
+      </c>
+      <c r="C10" s="5"/>
+      <c r="D10" s="3">
+        <v>0.67877864523998899</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3">
+        <v>0.72344901968392195</v>
+      </c>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
@@ -618,42 +626,6 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
@@ -670,6 +642,42 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="F7:G7"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
week 9 queries generated (1/2).
</commit_message>
<xml_diff>
--- a/Function 1/evals.xlsx
+++ b/Function 1/evals.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E37FB250-F364-4613-AFE8-D52D19B4C019}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB17A886-1DFC-4A81-8310-55A7E10B496A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -374,9 +374,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:M14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
@@ -396,7 +396,7 @@
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B3" s="5">
         <v>1</v>
       </c>
@@ -416,7 +416,7 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" s="5">
         <v>2</v>
       </c>
@@ -438,7 +438,7 @@
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B5" s="5">
         <v>3</v>
       </c>
@@ -460,7 +460,7 @@
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" s="5">
         <v>4</v>
       </c>
@@ -482,7 +482,7 @@
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7" s="5">
         <v>5</v>
       </c>
@@ -504,7 +504,7 @@
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="5">
         <v>6</v>
       </c>
@@ -526,7 +526,7 @@
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" s="5">
         <v>7</v>
       </c>
@@ -548,7 +548,7 @@
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
     </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B10" s="5">
         <v>8</v>
       </c>
@@ -561,19 +561,27 @@
         <v>0.72344901968392195</v>
       </c>
       <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
+      <c r="H10" s="4">
+        <v>6.2317929142213798E-9</v>
+      </c>
       <c r="I10" s="3"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B11" s="5">
+        <v>9</v>
+      </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="3">
+        <v>0.66863773391945702</v>
+      </c>
       <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
+      <c r="F11" s="3">
+        <v>0.72020275650301302</v>
+      </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -582,7 +590,7 @@
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -596,7 +604,7 @@
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
@@ -610,7 +618,7 @@
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>

</xml_diff>

<commit_message>
week 10 queries generated (1/2).
</commit_message>
<xml_diff>
--- a/Function 1/evals.xlsx
+++ b/Function 1/evals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB17A886-1DFC-4A81-8310-55A7E10B496A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D40F3F4-AED0-4CBA-B7F2-4F2F90455E75}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,13 +84,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -377,256 +377,268 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5" t="s">
+      <c r="E2" s="3"/>
+      <c r="F2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5" t="s">
+      <c r="G2" s="3"/>
+      <c r="H2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="5"/>
+      <c r="I2" s="3"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="5">
+      <c r="B3" s="3">
         <v>1</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="3">
+      <c r="C3" s="3"/>
+      <c r="D3" s="4">
         <v>0.73278699999999997</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3">
+      <c r="E3" s="4"/>
+      <c r="F3" s="4">
         <v>0.73318099999999997</v>
       </c>
-      <c r="G3" s="3"/>
-      <c r="H3" s="4">
+      <c r="G3" s="4"/>
+      <c r="H3" s="5">
         <v>3.5897238714370398E-16</v>
       </c>
-      <c r="I3" s="3"/>
+      <c r="I3" s="4"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="5">
+      <c r="B4" s="3">
         <v>2</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="3">
+      <c r="C4" s="3"/>
+      <c r="D4" s="4">
         <v>0.5</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3">
+      <c r="E4" s="4"/>
+      <c r="F4" s="4">
         <v>0.45</v>
       </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="4">
+      <c r="G4" s="4"/>
+      <c r="H4" s="5">
         <v>-5.8471552540567497E-6</v>
       </c>
-      <c r="I4" s="3"/>
+      <c r="I4" s="4"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="5">
+      <c r="B5" s="3">
         <v>3</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="3">
+      <c r="C5" s="3"/>
+      <c r="D5" s="4">
         <v>0.71610380492128201</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3">
+      <c r="E5" s="4"/>
+      <c r="F5" s="4">
         <v>0.73107980911083703</v>
       </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="4">
+      <c r="G5" s="4"/>
+      <c r="H5" s="5">
         <v>2.4917657838054898E-13</v>
       </c>
-      <c r="I5" s="3"/>
+      <c r="I5" s="4"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B6" s="5">
+      <c r="B6" s="3">
         <v>4</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="3">
+      <c r="C6" s="3"/>
+      <c r="D6" s="4">
         <v>0.70174915499430002</v>
       </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3">
+      <c r="E6" s="4"/>
+      <c r="F6" s="4">
         <v>0.72858430442151101</v>
       </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="4">
+      <c r="G6" s="4"/>
+      <c r="H6" s="5">
         <v>2.66967348318954E-11</v>
       </c>
-      <c r="I6" s="3"/>
+      <c r="I6" s="4"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="5">
+      <c r="B7" s="3">
         <v>5</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="3">
+      <c r="C7" s="3"/>
+      <c r="D7" s="4">
         <v>0.69774526461712905</v>
       </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3">
+      <c r="E7" s="4"/>
+      <c r="F7" s="4">
         <v>0.72787423209350399</v>
       </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="4">
+      <c r="G7" s="4"/>
+      <c r="H7" s="5">
         <v>8.2021938139919396E-11</v>
       </c>
-      <c r="I7" s="3"/>
+      <c r="I7" s="4"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="5">
+      <c r="B8" s="3">
         <v>6</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="3">
+      <c r="C8" s="3"/>
+      <c r="D8" s="4">
         <v>0.69108273489459604</v>
       </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3">
+      <c r="E8" s="4"/>
+      <c r="F8" s="4">
         <v>0.72641993605285105</v>
       </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="4">
+      <c r="G8" s="4"/>
+      <c r="H8" s="5">
         <v>4.8363240034292804E-10</v>
       </c>
-      <c r="I8" s="3"/>
+      <c r="I8" s="4"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="5">
+      <c r="B9" s="3">
         <v>7</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="3">
+      <c r="C9" s="3"/>
+      <c r="D9" s="4">
         <v>0.68231104396327502</v>
       </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3">
+      <c r="E9" s="4"/>
+      <c r="F9" s="4">
         <v>0.72440711698077198</v>
       </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="4">
+      <c r="G9" s="4"/>
+      <c r="H9" s="5">
         <v>3.3931989655218898E-9</v>
       </c>
-      <c r="I9" s="3"/>
+      <c r="I9" s="4"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="5">
+      <c r="B10" s="3">
         <v>8</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="3">
+      <c r="C10" s="3"/>
+      <c r="D10" s="4">
         <v>0.67877864523998899</v>
       </c>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3">
+      <c r="E10" s="4"/>
+      <c r="F10" s="4">
         <v>0.72344901968392195</v>
       </c>
-      <c r="G10" s="3"/>
-      <c r="H10" s="4">
+      <c r="G10" s="4"/>
+      <c r="H10" s="5">
         <v>6.2317929142213798E-9</v>
       </c>
-      <c r="I10" s="3"/>
+      <c r="I10" s="4"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="5">
+      <c r="B11" s="3">
         <v>9</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="3">
+      <c r="C11" s="3"/>
+      <c r="D11" s="4">
         <v>0.66863773391945702</v>
       </c>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3">
+      <c r="E11" s="4"/>
+      <c r="F11" s="4">
         <v>0.72020275650301302</v>
       </c>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="5">
+        <v>6.3491792111265201E-9</v>
+      </c>
+      <c r="I11" s="4"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="3"/>
+      <c r="B12" s="3">
+        <v>10</v>
+      </c>
       <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
+      <c r="D12" s="4">
+        <v>0.67803095631347499</v>
+      </c>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4">
+        <v>0.73817923173427002</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="3"/>
+      <c r="B13" s="3">
+        <v>11</v>
+      </c>
       <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="3"/>
+      <c r="B14" s="3">
+        <v>12</v>
+      </c>
       <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
@@ -634,6 +646,42 @@
     </row>
   </sheetData>
   <mergeCells count="52">
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
@@ -650,42 +698,6 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="F7:G7"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
generating week 11 queries (1/2)
</commit_message>
<xml_diff>
--- a/Function 1/evals.xlsx
+++ b/Function 1/evals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D40F3F4-AED0-4CBA-B7F2-4F2F90455E75}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37D37E4E-9096-4CC3-80F8-9180E8CEE911}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,13 +84,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -377,268 +377,274 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="5"/>
+      <c r="D2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
+      <c r="E2" s="5"/>
+      <c r="F2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3" t="s">
+      <c r="G2" s="5"/>
+      <c r="H2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="3"/>
+      <c r="I2" s="5"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="3">
+      <c r="B3" s="5">
         <v>1</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="4">
-        <v>0.73278699999999997</v>
-      </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4">
-        <v>0.73318099999999997</v>
-      </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="5">
+      <c r="C3" s="5"/>
+      <c r="D3" s="3">
+        <v>0.73278743099999999</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3">
+        <v>0.73318142100000006</v>
+      </c>
+      <c r="G3" s="3"/>
+      <c r="H3" s="4">
         <v>3.5897238714370398E-16</v>
       </c>
-      <c r="I3" s="4"/>
+      <c r="I3" s="3"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="3">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="4">
+      <c r="C4" s="5"/>
+      <c r="D4" s="3">
         <v>0.5</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4">
+      <c r="E4" s="3"/>
+      <c r="F4" s="3">
         <v>0.45</v>
       </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="5">
+      <c r="G4" s="3"/>
+      <c r="H4" s="4">
         <v>-5.8471552540567497E-6</v>
       </c>
-      <c r="I4" s="4"/>
+      <c r="I4" s="3"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="3">
+      <c r="B5" s="5">
         <v>3</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="4">
+      <c r="C5" s="5"/>
+      <c r="D5" s="3">
         <v>0.71610380492128201</v>
       </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4">
+      <c r="E5" s="3"/>
+      <c r="F5" s="3">
         <v>0.73107980911083703</v>
       </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="5">
+      <c r="G5" s="3"/>
+      <c r="H5" s="4">
         <v>2.4917657838054898E-13</v>
       </c>
-      <c r="I5" s="4"/>
+      <c r="I5" s="3"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B6" s="3">
+      <c r="B6" s="5">
         <v>4</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="4">
+      <c r="C6" s="5"/>
+      <c r="D6" s="3">
         <v>0.70174915499430002</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4">
+      <c r="E6" s="3"/>
+      <c r="F6" s="3">
         <v>0.72858430442151101</v>
       </c>
-      <c r="G6" s="4"/>
-      <c r="H6" s="5">
+      <c r="G6" s="3"/>
+      <c r="H6" s="4">
         <v>2.66967348318954E-11</v>
       </c>
-      <c r="I6" s="4"/>
+      <c r="I6" s="3"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="3">
+      <c r="B7" s="5">
         <v>5</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="4">
+      <c r="C7" s="5"/>
+      <c r="D7" s="3">
         <v>0.69774526461712905</v>
       </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4">
+      <c r="E7" s="3"/>
+      <c r="F7" s="3">
         <v>0.72787423209350399</v>
       </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="5">
+      <c r="G7" s="3"/>
+      <c r="H7" s="4">
         <v>8.2021938139919396E-11</v>
       </c>
-      <c r="I7" s="4"/>
+      <c r="I7" s="3"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="3">
+      <c r="B8" s="5">
         <v>6</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="4">
+      <c r="C8" s="5"/>
+      <c r="D8" s="3">
         <v>0.69108273489459604</v>
       </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4">
+      <c r="E8" s="3"/>
+      <c r="F8" s="3">
         <v>0.72641993605285105</v>
       </c>
-      <c r="G8" s="4"/>
-      <c r="H8" s="5">
+      <c r="G8" s="3"/>
+      <c r="H8" s="4">
         <v>4.8363240034292804E-10</v>
       </c>
-      <c r="I8" s="4"/>
+      <c r="I8" s="3"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="3">
+      <c r="B9" s="5">
         <v>7</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="4">
+      <c r="C9" s="5"/>
+      <c r="D9" s="3">
         <v>0.68231104396327502</v>
       </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4">
+      <c r="E9" s="3"/>
+      <c r="F9" s="3">
         <v>0.72440711698077198</v>
       </c>
-      <c r="G9" s="4"/>
-      <c r="H9" s="5">
+      <c r="G9" s="3"/>
+      <c r="H9" s="4">
         <v>3.3931989655218898E-9</v>
       </c>
-      <c r="I9" s="4"/>
+      <c r="I9" s="3"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="3">
+      <c r="B10" s="5">
         <v>8</v>
       </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="4">
+      <c r="C10" s="5"/>
+      <c r="D10" s="3">
         <v>0.67877864523998899</v>
       </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4">
+      <c r="E10" s="3"/>
+      <c r="F10" s="3">
         <v>0.72344901968392195</v>
       </c>
-      <c r="G10" s="4"/>
-      <c r="H10" s="5">
+      <c r="G10" s="3"/>
+      <c r="H10" s="4">
         <v>6.2317929142213798E-9</v>
       </c>
-      <c r="I10" s="4"/>
+      <c r="I10" s="3"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="3">
+      <c r="B11" s="5">
         <v>9</v>
       </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="4">
+      <c r="C11" s="5"/>
+      <c r="D11" s="3">
         <v>0.66863773391945702</v>
       </c>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4">
+      <c r="E11" s="3"/>
+      <c r="F11" s="3">
         <v>0.72020275650301302</v>
       </c>
-      <c r="G11" s="4"/>
-      <c r="H11" s="5">
+      <c r="G11" s="3"/>
+      <c r="H11" s="4">
         <v>6.3491792111265201E-9</v>
       </c>
-      <c r="I11" s="4"/>
+      <c r="I11" s="3"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="3">
+      <c r="B12" s="5">
         <v>10</v>
       </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="4">
+      <c r="C12" s="5"/>
+      <c r="D12" s="3">
         <v>0.67803095631347499</v>
       </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4">
+      <c r="E12" s="3"/>
+      <c r="F12" s="3">
         <v>0.73817923173427002</v>
       </c>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="4">
+        <v>2.2495964229471201E-11</v>
+      </c>
+      <c r="I12" s="3"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="3">
+      <c r="B13" s="5">
         <v>11</v>
       </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="3">
+        <v>0.67102657288577505</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3">
+        <v>0.72120796425721501</v>
+      </c>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="3">
+      <c r="B14" s="5">
         <v>12</v>
       </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
@@ -646,42 +652,6 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
@@ -698,6 +668,42 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="F7:G7"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
creating notebook for the generation of the query dataset.
</commit_message>
<xml_diff>
--- a/Function 1/evals.xlsx
+++ b/Function 1/evals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37D37E4E-9096-4CC3-80F8-9180E8CEE911}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F116B5A2-EB16-4AF5-8302-9DDE6E7BBEAC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
     <t>x2</t>
   </si>
   <si>
-    <t>f(x)</t>
+    <t>f(X)</t>
   </si>
 </sst>
 </file>
@@ -84,13 +84,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -377,274 +377,274 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5" t="s">
+      <c r="E2" s="3"/>
+      <c r="F2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5" t="s">
+      <c r="G2" s="3"/>
+      <c r="H2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="5"/>
+      <c r="I2" s="3"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="5">
+      <c r="B3" s="3">
         <v>1</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="3">
+      <c r="C3" s="3"/>
+      <c r="D3" s="4">
         <v>0.73278743099999999</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3">
+      <c r="E3" s="4"/>
+      <c r="F3" s="4">
         <v>0.73318142100000006</v>
       </c>
-      <c r="G3" s="3"/>
-      <c r="H3" s="4">
+      <c r="G3" s="4"/>
+      <c r="H3" s="5">
         <v>3.5897238714370398E-16</v>
       </c>
-      <c r="I3" s="3"/>
+      <c r="I3" s="4"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="5">
+      <c r="B4" s="3">
         <v>2</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="3">
+      <c r="C4" s="3"/>
+      <c r="D4" s="4">
         <v>0.5</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3">
+      <c r="E4" s="4"/>
+      <c r="F4" s="4">
         <v>0.45</v>
       </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="4">
+      <c r="G4" s="4"/>
+      <c r="H4" s="5">
         <v>-5.8471552540567497E-6</v>
       </c>
-      <c r="I4" s="3"/>
+      <c r="I4" s="4"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="5">
+      <c r="B5" s="3">
         <v>3</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="3">
+      <c r="C5" s="3"/>
+      <c r="D5" s="4">
         <v>0.71610380492128201</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3">
+      <c r="E5" s="4"/>
+      <c r="F5" s="4">
         <v>0.73107980911083703</v>
       </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="4">
+      <c r="G5" s="4"/>
+      <c r="H5" s="5">
         <v>2.4917657838054898E-13</v>
       </c>
-      <c r="I5" s="3"/>
+      <c r="I5" s="4"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B6" s="5">
+      <c r="B6" s="3">
         <v>4</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="3">
+      <c r="C6" s="3"/>
+      <c r="D6" s="4">
         <v>0.70174915499430002</v>
       </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3">
+      <c r="E6" s="4"/>
+      <c r="F6" s="4">
         <v>0.72858430442151101</v>
       </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="4">
+      <c r="G6" s="4"/>
+      <c r="H6" s="5">
         <v>2.66967348318954E-11</v>
       </c>
-      <c r="I6" s="3"/>
+      <c r="I6" s="4"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="5">
+      <c r="B7" s="3">
         <v>5</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="3">
+      <c r="C7" s="3"/>
+      <c r="D7" s="4">
         <v>0.69774526461712905</v>
       </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3">
+      <c r="E7" s="4"/>
+      <c r="F7" s="4">
         <v>0.72787423209350399</v>
       </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="4">
+      <c r="G7" s="4"/>
+      <c r="H7" s="5">
         <v>8.2021938139919396E-11</v>
       </c>
-      <c r="I7" s="3"/>
+      <c r="I7" s="4"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="5">
+      <c r="B8" s="3">
         <v>6</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="3">
+      <c r="C8" s="3"/>
+      <c r="D8" s="4">
         <v>0.69108273489459604</v>
       </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3">
+      <c r="E8" s="4"/>
+      <c r="F8" s="4">
         <v>0.72641993605285105</v>
       </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="4">
+      <c r="G8" s="4"/>
+      <c r="H8" s="5">
         <v>4.8363240034292804E-10</v>
       </c>
-      <c r="I8" s="3"/>
+      <c r="I8" s="4"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="5">
+      <c r="B9" s="3">
         <v>7</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="3">
+      <c r="C9" s="3"/>
+      <c r="D9" s="4">
         <v>0.68231104396327502</v>
       </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3">
+      <c r="E9" s="4"/>
+      <c r="F9" s="4">
         <v>0.72440711698077198</v>
       </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="4">
+      <c r="G9" s="4"/>
+      <c r="H9" s="5">
         <v>3.3931989655218898E-9</v>
       </c>
-      <c r="I9" s="3"/>
+      <c r="I9" s="4"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="5">
+      <c r="B10" s="3">
         <v>8</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="3">
+      <c r="C10" s="3"/>
+      <c r="D10" s="4">
         <v>0.67877864523998899</v>
       </c>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3">
+      <c r="E10" s="4"/>
+      <c r="F10" s="4">
         <v>0.72344901968392195</v>
       </c>
-      <c r="G10" s="3"/>
-      <c r="H10" s="4">
+      <c r="G10" s="4"/>
+      <c r="H10" s="5">
         <v>6.2317929142213798E-9</v>
       </c>
-      <c r="I10" s="3"/>
+      <c r="I10" s="4"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="5">
+      <c r="B11" s="3">
         <v>9</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="3">
+      <c r="C11" s="3"/>
+      <c r="D11" s="4">
         <v>0.66863773391945702</v>
       </c>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3">
+      <c r="E11" s="4"/>
+      <c r="F11" s="4">
         <v>0.72020275650301302</v>
       </c>
-      <c r="G11" s="3"/>
-      <c r="H11" s="4">
+      <c r="G11" s="4"/>
+      <c r="H11" s="5">
         <v>6.3491792111265201E-9</v>
       </c>
-      <c r="I11" s="3"/>
+      <c r="I11" s="4"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="5">
+      <c r="B12" s="3">
         <v>10</v>
       </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="3">
+      <c r="C12" s="3"/>
+      <c r="D12" s="4">
         <v>0.67803095631347499</v>
       </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3">
+      <c r="E12" s="4"/>
+      <c r="F12" s="4">
         <v>0.73817923173427002</v>
       </c>
-      <c r="G12" s="3"/>
-      <c r="H12" s="4">
+      <c r="G12" s="4"/>
+      <c r="H12" s="5">
         <v>2.2495964229471201E-11</v>
       </c>
-      <c r="I12" s="3"/>
+      <c r="I12" s="4"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="5">
+      <c r="B13" s="3">
         <v>11</v>
       </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="3">
+      <c r="C13" s="3"/>
+      <c r="D13" s="4">
         <v>0.67102657288577505</v>
       </c>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3">
+      <c r="E13" s="4"/>
+      <c r="F13" s="4">
         <v>0.72120796425721501</v>
       </c>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="5">
+      <c r="B14" s="3">
         <v>12</v>
       </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
@@ -652,6 +652,42 @@
     </row>
   </sheetData>
   <mergeCells count="52">
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
@@ -668,42 +704,6 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="F7:G7"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
week 12 queries generated and submitted.
</commit_message>
<xml_diff>
--- a/Function 1/evals.xlsx
+++ b/Function 1/evals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prithvi\Desktop\Imperial Course\Capstone-Project\Function 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F116B5A2-EB16-4AF5-8302-9DDE6E7BBEAC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF065423-B210-4306-B691-285D25191ABA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,13 +84,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -373,34 +373,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:M14"/>
+  <dimension ref="B2:M15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="5"/>
+      <c r="D2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
+      <c r="E2" s="5"/>
+      <c r="F2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3" t="s">
+      <c r="G2" s="5"/>
+      <c r="H2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="3"/>
+      <c r="I2" s="5"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="3">
+      <c r="B3" s="5">
         <v>1</v>
       </c>
-      <c r="C3" s="3"/>
+      <c r="C3" s="5"/>
       <c r="D3" s="4">
         <v>0.73278743099999999</v>
       </c>
@@ -409,7 +409,7 @@
         <v>0.73318142100000006</v>
       </c>
       <c r="G3" s="4"/>
-      <c r="H3" s="5">
+      <c r="H3" s="3">
         <v>3.5897238714370398E-16</v>
       </c>
       <c r="I3" s="4"/>
@@ -417,10 +417,10 @@
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="3">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="3"/>
+      <c r="C4" s="5"/>
       <c r="D4" s="4">
         <v>0.5</v>
       </c>
@@ -429,7 +429,7 @@
         <v>0.45</v>
       </c>
       <c r="G4" s="4"/>
-      <c r="H4" s="5">
+      <c r="H4" s="3">
         <v>-5.8471552540567497E-6</v>
       </c>
       <c r="I4" s="4"/>
@@ -439,10 +439,10 @@
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="3">
+      <c r="B5" s="5">
         <v>3</v>
       </c>
-      <c r="C5" s="3"/>
+      <c r="C5" s="5"/>
       <c r="D5" s="4">
         <v>0.71610380492128201</v>
       </c>
@@ -451,7 +451,7 @@
         <v>0.73107980911083703</v>
       </c>
       <c r="G5" s="4"/>
-      <c r="H5" s="5">
+      <c r="H5" s="3">
         <v>2.4917657838054898E-13</v>
       </c>
       <c r="I5" s="4"/>
@@ -461,10 +461,10 @@
       <c r="M5" s="1"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B6" s="3">
+      <c r="B6" s="5">
         <v>4</v>
       </c>
-      <c r="C6" s="3"/>
+      <c r="C6" s="5"/>
       <c r="D6" s="4">
         <v>0.70174915499430002</v>
       </c>
@@ -473,7 +473,7 @@
         <v>0.72858430442151101</v>
       </c>
       <c r="G6" s="4"/>
-      <c r="H6" s="5">
+      <c r="H6" s="3">
         <v>2.66967348318954E-11</v>
       </c>
       <c r="I6" s="4"/>
@@ -483,10 +483,10 @@
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="3">
+      <c r="B7" s="5">
         <v>5</v>
       </c>
-      <c r="C7" s="3"/>
+      <c r="C7" s="5"/>
       <c r="D7" s="4">
         <v>0.69774526461712905</v>
       </c>
@@ -495,7 +495,7 @@
         <v>0.72787423209350399</v>
       </c>
       <c r="G7" s="4"/>
-      <c r="H7" s="5">
+      <c r="H7" s="3">
         <v>8.2021938139919396E-11</v>
       </c>
       <c r="I7" s="4"/>
@@ -505,10 +505,10 @@
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="3">
+      <c r="B8" s="5">
         <v>6</v>
       </c>
-      <c r="C8" s="3"/>
+      <c r="C8" s="5"/>
       <c r="D8" s="4">
         <v>0.69108273489459604</v>
       </c>
@@ -517,7 +517,7 @@
         <v>0.72641993605285105</v>
       </c>
       <c r="G8" s="4"/>
-      <c r="H8" s="5">
+      <c r="H8" s="3">
         <v>4.8363240034292804E-10</v>
       </c>
       <c r="I8" s="4"/>
@@ -527,10 +527,10 @@
       <c r="M8" s="1"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="3">
+      <c r="B9" s="5">
         <v>7</v>
       </c>
-      <c r="C9" s="3"/>
+      <c r="C9" s="5"/>
       <c r="D9" s="4">
         <v>0.68231104396327502</v>
       </c>
@@ -539,7 +539,7 @@
         <v>0.72440711698077198</v>
       </c>
       <c r="G9" s="4"/>
-      <c r="H9" s="5">
+      <c r="H9" s="3">
         <v>3.3931989655218898E-9</v>
       </c>
       <c r="I9" s="4"/>
@@ -549,10 +549,10 @@
       <c r="M9" s="1"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="3">
+      <c r="B10" s="5">
         <v>8</v>
       </c>
-      <c r="C10" s="3"/>
+      <c r="C10" s="5"/>
       <c r="D10" s="4">
         <v>0.67877864523998899</v>
       </c>
@@ -561,7 +561,7 @@
         <v>0.72344901968392195</v>
       </c>
       <c r="G10" s="4"/>
-      <c r="H10" s="5">
+      <c r="H10" s="3">
         <v>6.2317929142213798E-9</v>
       </c>
       <c r="I10" s="4"/>
@@ -571,10 +571,10 @@
       <c r="M10" s="1"/>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="3">
+      <c r="B11" s="5">
         <v>9</v>
       </c>
-      <c r="C11" s="3"/>
+      <c r="C11" s="5"/>
       <c r="D11" s="4">
         <v>0.66863773391945702</v>
       </c>
@@ -583,7 +583,7 @@
         <v>0.72020275650301302</v>
       </c>
       <c r="G11" s="4"/>
-      <c r="H11" s="5">
+      <c r="H11" s="3">
         <v>6.3491792111265201E-9</v>
       </c>
       <c r="I11" s="4"/>
@@ -593,10 +593,10 @@
       <c r="M11" s="1"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="3">
+      <c r="B12" s="5">
         <v>10</v>
       </c>
-      <c r="C12" s="3"/>
+      <c r="C12" s="5"/>
       <c r="D12" s="4">
         <v>0.67803095631347499</v>
       </c>
@@ -605,7 +605,7 @@
         <v>0.73817923173427002</v>
       </c>
       <c r="G12" s="4"/>
-      <c r="H12" s="5">
+      <c r="H12" s="3">
         <v>2.2495964229471201E-11</v>
       </c>
       <c r="I12" s="4"/>
@@ -615,10 +615,10 @@
       <c r="M12" s="1"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="3">
+      <c r="B13" s="5">
         <v>11</v>
       </c>
-      <c r="C13" s="3"/>
+      <c r="C13" s="5"/>
       <c r="D13" s="4">
         <v>0.67102657288577505</v>
       </c>
@@ -627,7 +627,9 @@
         <v>0.72120796425721501</v>
       </c>
       <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
+      <c r="H13" s="3">
+        <v>1.30167165987852E-8</v>
+      </c>
       <c r="I13" s="4"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
@@ -635,13 +637,17 @@
       <c r="M13" s="1"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="3">
+      <c r="B14" s="5">
         <v>12</v>
       </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="4"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="4">
+        <v>0.66951685761810298</v>
+      </c>
       <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
+      <c r="F14" s="4">
+        <v>0.72297880096555001</v>
+      </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
@@ -650,44 +656,24 @@
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
     </row>
+    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B15" s="5">
+        <v>13</v>
+      </c>
+      <c r="C15" s="5"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+    </row>
   </sheetData>
-  <mergeCells count="52">
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
+  <mergeCells count="56">
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="H15:I15"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
@@ -704,6 +690,42 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="F7:G7"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F12:G12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>